<commit_message>
Add comments to the C# wrapper
CommentEntry mirroring the F# core's own CommentEntry exactly, plus
Sheet.WithComments/AddComment. Author defaults to "", matching how Excel
itself allows an unnamed comment author. Reconstructs the F# Worksheet's
Comments field the same way hyperlinks/data validations already do -
baseline via sheetOfCells, override just the fields this wrapper models.

Updated CsCodeGen for the new type before writing tests, same discipline
established after the sparklines gap. RenderCommentEntry omits the
author argument entirely when it's empty, matching CommentEntry.Of's own
default.

4 new tests (92 total): an Examples/ scenario mirroring the F# suite's
own Comments scenario exactly (three comments, two authored and one not,
verified to actually execute via `dotnet run`), plus unit tests for
defaults/immutability.

Updated the wrapper's README and llms.txt - comments moves from "not
exposed" to "covers".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.CsOpenXmlDsl.Tests/Examples/ChartBar/output.xlsx
+++ b/tests/Kookerella.CsOpenXmlDsl.Tests/Examples/ChartBar/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2b5625a65b7046b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R09e2e1e2dfeb4095"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb8526d2ca62a41f4"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R2b43d8619639407c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -177,6 +177,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf49194423ab4c7c"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc11992396bc7478f"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add sheet and workbook protection to the C# wrapper
Adds SheetProtection/WorkbookProtection, closing out the last remaining
feature-parity gap between the C# wrapper and the F# core (everything
except per-cell lock/hide protection is now covered). SheetProtection's
optional flags carry a deliberate Blocked suffix (FormatCellsBlocked,
SortBlocked, ...) rather than mirroring the F# field names verbatim, to
avoid the F# core's inverted-meaning footgun where e.g. FormatCells =
true means formatting becomes blocked, not enabled.

Also fixes a staleness gap in AssertWorkbooksMatch, which had not been
updated since sparklines and was silently skipping round-trip
verification for five-plus later features in the slow example-script
test suite.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.CsOpenXmlDsl.Tests/Examples/ChartBar/output.xlsx
+++ b/tests/Kookerella.CsOpenXmlDsl.Tests/Examples/ChartBar/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rd721fc6c4d654c12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7ed1ff95558c4f37"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R3f1b2ea3b6714352"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Radee52537b0b4472"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -177,6 +177,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5805565ed1254274"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc912b62ea3dd47ca"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add per-cell lock/hide protection to the C# wrapper
Adds CellProtection (Locked/Hidden) on CellStyle, closing the last
remaining feature gap between the C# wrapper and the F# core - the
wrapper now has full parity. Locked/Hidden mirror the F# field names
directly since neither carries the inverted-meaning trap that motivated
SheetProtection's Blocked-suffix naming.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.CsOpenXmlDsl.Tests/Examples/ChartBar/output.xlsx
+++ b/tests/Kookerella.CsOpenXmlDsl.Tests/Examples/ChartBar/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R7ed1ff95558c4f37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R53a8adebe18d4e27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Radee52537b0b4472"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rff21e4aaf64c46cc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -177,6 +177,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc912b62ea3dd47ca"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf54391fe7fe54963"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Bump Kookerella.FsOpenXmlDsl to 0.2.0 for the new Xml module
The published package was still at 0.1.2, from before Xml.fs/Xml.xsd
existed - anyone installing it directly from NuGet got none of the
XML interpreter work. The Mcp server was unaffected only because it
builds against local source via ProjectReference, which masked the
gap. Description updated to mention the XML surface and its two uses
(building from XSLT-generated XML, converting to XML for git-diffable
version control).

Packed via `dotnet fake run build.fsx -t PackCore`, which runs the
full fast+slow test gate (F# and C# wrapper) before producing the
package - the first real use of build.fsx for an actual release
rather than manual dotnet pack.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/Kookerella.CsOpenXmlDsl.Tests/Examples/ChartBar/output.xlsx
+++ b/tests/Kookerella.CsOpenXmlDsl.Tests/Examples/ChartBar/output.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6af08a1afcd74d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra4ceb86ff7054c83"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -140,7 +140,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R944cf4ceaf594a62"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R676fa4782ed749be"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -177,6 +177,6 @@
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reda829614f6e4de5"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra48185f01ac74e35"/>
 </x:worksheet>
 </file>
</xml_diff>